<commit_message>
Fix URL rule to split houses and apartments
</commit_message>
<xml_diff>
--- a/data/CHI_SO_PHAI_SINH.xlsx
+++ b/data/CHI_SO_PHAI_SINH.xlsx
@@ -4912,7 +4912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1441"/>
+  <dimension ref="A1:N1457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -73024,6 +73024,774 @@
         <v>0</v>
       </c>
       <c r="N1441" s="6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1442" s="3" t="inlineStr">
+        <is>
+          <t>Nam Từ Liêm</t>
+        </is>
+      </c>
+      <c r="C1442" s="4" t="n">
+        <v>4915</v>
+      </c>
+      <c r="D1442" s="4" t="n">
+        <v>18677</v>
+      </c>
+      <c r="E1442" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F1442" s="4" t="n">
+        <v>172</v>
+      </c>
+      <c r="G1442" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1442" s="4" t="n">
+        <v>376</v>
+      </c>
+      <c r="I1442" s="4" t="n">
+        <v>210.1</v>
+      </c>
+      <c r="J1442" s="4" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="K1442" s="4" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="L1442" s="4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="M1442" s="4" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="N1442" s="4" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1443" s="5" t="inlineStr">
+        <is>
+          <t>Cầu Giấy</t>
+        </is>
+      </c>
+      <c r="C1443" s="6" t="n">
+        <v>4909</v>
+      </c>
+      <c r="D1443" s="6" t="n">
+        <v>30927</v>
+      </c>
+      <c r="E1443" s="6" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F1443" s="6" t="n">
+        <v>135.4</v>
+      </c>
+      <c r="G1443" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1443" s="6" t="n">
+        <v>567</v>
+      </c>
+      <c r="I1443" s="6" t="n">
+        <v>338.6</v>
+      </c>
+      <c r="J1443" s="6" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="K1443" s="6" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="L1443" s="6" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="M1443" s="6" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="N1443" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1444" s="3" t="inlineStr">
+        <is>
+          <t>Hà Đông</t>
+        </is>
+      </c>
+      <c r="C1444" s="4" t="n">
+        <v>5774</v>
+      </c>
+      <c r="D1444" s="4" t="n">
+        <v>34067</v>
+      </c>
+      <c r="E1444" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F1444" s="4" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="G1444" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="H1444" s="4" t="n">
+        <v>642</v>
+      </c>
+      <c r="I1444" s="4" t="n">
+        <v>403</v>
+      </c>
+      <c r="J1444" s="4" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="K1444" s="4" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="L1444" s="4" t="n">
+        <v>-20.2</v>
+      </c>
+      <c r="M1444" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N1444" s="4" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1445" s="5" t="inlineStr">
+        <is>
+          <t>Hoàng Mai</t>
+        </is>
+      </c>
+      <c r="C1445" s="6" t="n">
+        <v>3867</v>
+      </c>
+      <c r="D1445" s="6" t="n">
+        <v>23975</v>
+      </c>
+      <c r="E1445" s="6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F1445" s="6" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="G1445" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="H1445" s="6" t="n">
+        <v>712</v>
+      </c>
+      <c r="I1445" s="6" t="n">
+        <v>347.4</v>
+      </c>
+      <c r="J1445" s="6" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="K1445" s="6" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="L1445" s="6" t="n">
+        <v>-30.8</v>
+      </c>
+      <c r="M1445" s="6" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="N1445" s="6" t="n">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1446" s="3" t="inlineStr">
+        <is>
+          <t>Thanh Xuân</t>
+        </is>
+      </c>
+      <c r="C1446" s="4" t="n">
+        <v>3388</v>
+      </c>
+      <c r="D1446" s="4" t="n">
+        <v>24055</v>
+      </c>
+      <c r="E1446" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F1446" s="4" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="G1446" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="H1446" s="4" t="n">
+        <v>561</v>
+      </c>
+      <c r="I1446" s="4" t="n">
+        <v>264.6</v>
+      </c>
+      <c r="J1446" s="4" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="K1446" s="4" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="L1446" s="4" t="n">
+        <v>-18.9</v>
+      </c>
+      <c r="M1446" s="4" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="N1446" s="4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1447" s="5" t="inlineStr">
+        <is>
+          <t>Tây Hồ</t>
+        </is>
+      </c>
+      <c r="C1447" s="6" t="n">
+        <v>3093</v>
+      </c>
+      <c r="D1447" s="6" t="n">
+        <v>16702</v>
+      </c>
+      <c r="E1447" s="6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F1447" s="6" t="n">
+        <v>202.8</v>
+      </c>
+      <c r="G1447" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="H1447" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="I1447" s="6" t="n">
+        <v>180.7</v>
+      </c>
+      <c r="J1447" s="6" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="K1447" s="6" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L1447" s="6" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="M1447" s="6" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="N1447" s="6" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1448" s="3" t="inlineStr">
+        <is>
+          <t>Bắc Từ Liêm</t>
+        </is>
+      </c>
+      <c r="C1448" s="4" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D1448" s="4" t="n">
+        <v>17430</v>
+      </c>
+      <c r="E1448" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1448" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="G1448" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="H1448" s="4" t="n">
+        <v>484</v>
+      </c>
+      <c r="I1448" s="4" t="n">
+        <v>200.4</v>
+      </c>
+      <c r="J1448" s="4" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="K1448" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L1448" s="4" t="n">
+        <v>-32</v>
+      </c>
+      <c r="M1448" s="4" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="N1448" s="4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1449" s="5" t="inlineStr">
+        <is>
+          <t>Gia Lâm</t>
+        </is>
+      </c>
+      <c r="C1449" s="6" t="n">
+        <v>2142</v>
+      </c>
+      <c r="D1449" s="6" t="n">
+        <v>8782</v>
+      </c>
+      <c r="E1449" s="6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F1449" s="6" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="G1449" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1449" s="6" t="n">
+        <v>303</v>
+      </c>
+      <c r="I1449" s="6" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="J1449" s="6" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="K1449" s="6" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="L1449" s="6" t="n">
+        <v>-50.6</v>
+      </c>
+      <c r="M1449" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="N1449" s="6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1450" s="3" t="inlineStr">
+        <is>
+          <t>Long Biên</t>
+        </is>
+      </c>
+      <c r="C1450" s="4" t="n">
+        <v>4044</v>
+      </c>
+      <c r="D1450" s="4" t="n">
+        <v>34778</v>
+      </c>
+      <c r="E1450" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F1450" s="4" t="n">
+        <v>195.2</v>
+      </c>
+      <c r="G1450" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="H1450" s="4" t="n">
+        <v>790</v>
+      </c>
+      <c r="I1450" s="4" t="n">
+        <v>445.2</v>
+      </c>
+      <c r="J1450" s="4" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="K1450" s="4" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="L1450" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="M1450" s="4" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="N1450" s="4" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1451" s="5" t="inlineStr">
+        <is>
+          <t>Hoài Đức</t>
+        </is>
+      </c>
+      <c r="C1451" s="6" t="n">
+        <v>2418</v>
+      </c>
+      <c r="D1451" s="6" t="n">
+        <v>15233</v>
+      </c>
+      <c r="E1451" s="6" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F1451" s="6" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="G1451" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="H1451" s="6" t="n">
+        <v>531</v>
+      </c>
+      <c r="I1451" s="6" t="n">
+        <v>204.1</v>
+      </c>
+      <c r="J1451" s="6" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="K1451" s="6" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="L1451" s="6" t="n">
+        <v>-45.2</v>
+      </c>
+      <c r="M1451" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N1451" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1452" s="3" t="inlineStr">
+        <is>
+          <t>Đống Đa</t>
+        </is>
+      </c>
+      <c r="C1452" s="4" t="n">
+        <v>3288</v>
+      </c>
+      <c r="D1452" s="4" t="n">
+        <v>32880</v>
+      </c>
+      <c r="E1452" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1452" s="4" t="n">
+        <v>262.5</v>
+      </c>
+      <c r="G1452" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1452" s="4" t="n">
+        <v>693</v>
+      </c>
+      <c r="I1452" s="4" t="n">
+        <v>353.5</v>
+      </c>
+      <c r="J1452" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="K1452" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1452" s="4" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="M1452" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N1452" s="4" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1453" s="5" t="inlineStr">
+        <is>
+          <t>Hai Bà Trưng</t>
+        </is>
+      </c>
+      <c r="C1453" s="6" t="n">
+        <v>2226</v>
+      </c>
+      <c r="D1453" s="6" t="n">
+        <v>22928</v>
+      </c>
+      <c r="E1453" s="6" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F1453" s="6" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="G1453" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1453" s="6" t="n">
+        <v>593</v>
+      </c>
+      <c r="I1453" s="6" t="n">
+        <v>247.6</v>
+      </c>
+      <c r="J1453" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="K1453" s="6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="L1453" s="6" t="n">
+        <v>-18</v>
+      </c>
+      <c r="M1453" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="N1453" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1454" s="3" t="inlineStr">
+        <is>
+          <t>Thanh Trì</t>
+        </is>
+      </c>
+      <c r="C1454" s="4" t="n">
+        <v>1074</v>
+      </c>
+      <c r="D1454" s="4" t="n">
+        <v>10310</v>
+      </c>
+      <c r="E1454" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F1454" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="G1454" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="H1454" s="4" t="n">
+        <v>610</v>
+      </c>
+      <c r="I1454" s="4" t="n">
+        <v>148.6</v>
+      </c>
+      <c r="J1454" s="4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="K1454" s="4" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L1454" s="4" t="n">
+        <v>-9.1</v>
+      </c>
+      <c r="M1454" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N1454" s="4" t="n">
+        <v>44.1</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1455" s="5" t="inlineStr">
+        <is>
+          <t>Ba Đình</t>
+        </is>
+      </c>
+      <c r="C1455" s="6" t="n">
+        <v>2096</v>
+      </c>
+      <c r="D1455" s="6" t="n">
+        <v>19912</v>
+      </c>
+      <c r="E1455" s="6" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F1455" s="6" t="n">
+        <v>226.4</v>
+      </c>
+      <c r="G1455" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="H1455" s="6" t="n">
+        <v>530</v>
+      </c>
+      <c r="I1455" s="6" t="n">
+        <v>211.1</v>
+      </c>
+      <c r="J1455" s="6" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="K1455" s="6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L1455" s="6" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="M1455" s="6" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="N1455" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1456" s="3" t="inlineStr">
+        <is>
+          <t>Đông Anh</t>
+        </is>
+      </c>
+      <c r="C1456" s="4" t="n">
+        <v>1760</v>
+      </c>
+      <c r="D1456" s="4" t="n">
+        <v>17248</v>
+      </c>
+      <c r="E1456" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F1456" s="4" t="n">
+        <v>166.7</v>
+      </c>
+      <c r="G1456" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="H1456" s="4" t="n">
+        <v>653</v>
+      </c>
+      <c r="I1456" s="4" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="J1456" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="K1456" s="4" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="L1456" s="4" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="M1456" s="4" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="N1456" s="4" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1457" s="5" t="inlineStr">
+        <is>
+          <t>Đan Phượng</t>
+        </is>
+      </c>
+      <c r="C1457" s="6" t="n">
+        <v>721</v>
+      </c>
+      <c r="D1457" s="6" t="n">
+        <v>2668</v>
+      </c>
+      <c r="E1457" s="6" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F1457" s="6" t="n">
+        <v>160.2</v>
+      </c>
+      <c r="G1457" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="H1457" s="6" t="n">
+        <v>307</v>
+      </c>
+      <c r="I1457" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1457" s="6" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="K1457" s="6" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="L1457" s="6" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="M1457" s="6" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="N1457" s="6" t="n">
         <v>50</v>
       </c>
     </row>
@@ -73348,16 +74116,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3858</v>
+        <v>4044</v>
       </c>
       <c r="C16" t="n">
-        <v>37808</v>
+        <v>34778</v>
       </c>
       <c r="D16" t="n">
-        <v>9.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="E16" t="n">
-        <v>250.7</v>
+        <v>195.2</v>
       </c>
     </row>
   </sheetData>
@@ -73682,16 +74450,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4694</v>
+        <v>4915</v>
       </c>
       <c r="C16" t="n">
-        <v>18776</v>
+        <v>18677</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="E16" t="n">
-        <v>133.8</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -74016,16 +74784,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1214</v>
+        <v>1074</v>
       </c>
       <c r="C16" t="n">
-        <v>11776</v>
+        <v>10310</v>
       </c>
       <c r="D16" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="E16" t="n">
-        <v>130.9</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -74350,16 +75118,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3403</v>
+        <v>3388</v>
       </c>
       <c r="C16" t="n">
-        <v>23481</v>
+        <v>24055</v>
       </c>
       <c r="D16" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="E16" t="n">
-        <v>161.6</v>
+        <v>120.4</v>
       </c>
     </row>
   </sheetData>
@@ -74684,16 +75452,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2971</v>
+        <v>3093</v>
       </c>
       <c r="C16" t="n">
-        <v>16340</v>
+        <v>16702</v>
       </c>
       <c r="D16" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="E16" t="n">
-        <v>261</v>
+        <v>202.8</v>
       </c>
     </row>
   </sheetData>
@@ -75018,16 +75786,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>721</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>2668</v>
       </c>
       <c r="D16" t="n">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>160.2</v>
       </c>
     </row>
   </sheetData>
@@ -75352,16 +76120,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1867</v>
+        <v>1760</v>
       </c>
       <c r="C16" t="n">
-        <v>19043</v>
+        <v>17248</v>
       </c>
       <c r="D16" t="n">
-        <v>10.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>203.7</v>
+        <v>166.7</v>
       </c>
     </row>
   </sheetData>
@@ -75686,16 +76454,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3179</v>
+        <v>3288</v>
       </c>
       <c r="C16" t="n">
-        <v>32744</v>
+        <v>32880</v>
       </c>
       <c r="D16" t="n">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>237.6</v>
+        <v>262.5</v>
       </c>
     </row>
   </sheetData>
@@ -76020,16 +76788,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2165</v>
+        <v>2096</v>
       </c>
       <c r="C16" t="n">
-        <v>23815</v>
+        <v>19912</v>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="E16" t="n">
-        <v>238.3</v>
+        <v>226.4</v>
       </c>
     </row>
   </sheetData>
@@ -76354,16 +77122,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2420</v>
+        <v>2490</v>
       </c>
       <c r="C16" t="n">
-        <v>16698</v>
+        <v>17430</v>
       </c>
       <c r="D16" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>122.8</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -76688,16 +77456,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>4909</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>30927</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>135.4</v>
       </c>
     </row>
   </sheetData>
@@ -77022,16 +77790,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2058</v>
+        <v>2142</v>
       </c>
       <c r="C16" t="n">
-        <v>10290</v>
+        <v>8782</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>4.1</v>
       </c>
       <c r="E16" t="n">
-        <v>130.7</v>
+        <v>73.3</v>
       </c>
     </row>
   </sheetData>
@@ -77356,16 +78124,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2266</v>
+        <v>2226</v>
       </c>
       <c r="C16" t="n">
-        <v>23793</v>
+        <v>22928</v>
       </c>
       <c r="D16" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="E16" t="n">
-        <v>153.5</v>
+        <v>121.8</v>
       </c>
     </row>
   </sheetData>
@@ -77690,16 +78458,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2618</v>
+        <v>2418</v>
       </c>
       <c r="C16" t="n">
-        <v>16755</v>
+        <v>15233</v>
       </c>
       <c r="D16" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="E16" t="n">
-        <v>146.2</v>
+        <v>81.40000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -78024,16 +78792,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3845</v>
+        <v>3867</v>
       </c>
       <c r="C16" t="n">
-        <v>24224</v>
+        <v>23975</v>
       </c>
       <c r="D16" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="E16" t="n">
-        <v>232.9</v>
+        <v>102.7</v>
       </c>
     </row>
   </sheetData>
@@ -78358,16 +79126,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>5774</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>34067</v>
       </c>
       <c r="D16" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>118.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>